<commit_message>
stap 7 van de opdragt gemaakt/aangepast
</commit_message>
<xml_diff>
--- a/Naomi/Week 6/Logboek.xlsx
+++ b/Naomi/Week 6/Logboek.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gebruiker\source\repos\DEAI_portfolio\DE samenwerken\Week 6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gebruiker\source\repos\DEAI_portfolio\Naomi\Week 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F9A25DF-3410-4EA4-812F-031E3096016C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD529573-2FE0-4175-8E22-F3C5072CA328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12000" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="30">
   <si>
     <t>Features</t>
   </si>
@@ -61,6 +61,61 @@
   </si>
   <si>
     <t>Neighborhood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>LinearRegression</t>
+  </si>
+  <si>
+    <t>SGDRegressor</t>
+  </si>
+  <si>
+    <t>max_iter = 1000</t>
+  </si>
+  <si>
+    <t>eta0 = 0.01</t>
+  </si>
+  <si>
+    <t>Preprocessing</t>
+  </si>
+  <si>
+    <t>MSE: 1546445122.0290785</t>
+  </si>
+  <si>
+    <t>R2: 0.8071174459628098</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>StandardScaler</t>
+  </si>
+  <si>
+    <t>max_iter = 2000</t>
+  </si>
+  <si>
+    <t>eta0 = 0.001</t>
+  </si>
+  <si>
+    <t>MSE: 1525163556.5752804</t>
+  </si>
+  <si>
+    <t>R2: 0.809771819299545</t>
+  </si>
+  <si>
+    <t>Year Built</t>
+  </si>
+  <si>
+    <t>MSE: 1497106037.8897483</t>
+  </si>
+  <si>
+    <t>R2: 0.8132713329821972</t>
   </si>
 </sst>
 </file>
@@ -96,13 +151,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -116,13 +184,69 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CC9D797F-4CED-4B4A-B6E9-41FB7C35005D}" name="Tabel1" displayName="Tabel1" ref="A1:D4" totalsRowShown="0">
-  <autoFilter ref="A1:D4" xr:uid="{CC9D797F-4CED-4B4A-B6E9-41FB7C35005D}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CC9D797F-4CED-4B4A-B6E9-41FB7C35005D}" name="Tabel1" displayName="Tabel1" ref="B2:F5" totalsRowShown="0">
+  <autoFilter ref="B2:F5" xr:uid="{CC9D797F-4CED-4B4A-B6E9-41FB7C35005D}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{0904ECDB-157B-4BDD-BB62-014B67DA9584}" name="Target"/>
     <tableColumn id="2" xr3:uid="{567C2AB2-970A-40C9-B710-732F559D5C69}" name="Features"/>
     <tableColumn id="3" xr3:uid="{4BAC2826-D838-40B2-AA58-BFDA5E3D29EB}" name="Hyperparamaters"/>
     <tableColumn id="4" xr3:uid="{66B9318C-2084-4A10-8CE7-ADE5D922275B}" name="Resultaten"/>
+    <tableColumn id="5" xr3:uid="{95B40B0B-D496-4CA2-8696-290BD5DB79B7}" name="Model"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4D3ACD67-2EF4-4780-A037-9BF618BDEB3B}" name="Tabel2" displayName="Tabel2" ref="B6:G9" totalsRowShown="0">
+  <autoFilter ref="B6:G9" xr:uid="{4D3ACD67-2EF4-4780-A037-9BF618BDEB3B}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{A60D7DA5-6560-4FCE-A025-43931F33FB65}" name="Target"/>
+    <tableColumn id="2" xr3:uid="{EBA708CE-376D-496E-BC90-62CAC577A420}" name="Features"/>
+    <tableColumn id="3" xr3:uid="{D8B4B5C6-7F47-4CA3-9137-AF39382C2CD3}" name="Hyperparamaters"/>
+    <tableColumn id="4" xr3:uid="{BE838798-3C9E-4175-B8E6-EEB45E97C44A}" name="Resultaten"/>
+    <tableColumn id="5" xr3:uid="{121165DA-3996-4D00-AA96-FB13B7E7C4BF}" name="Model"/>
+    <tableColumn id="6" xr3:uid="{7F8985BF-2358-4D09-97F5-0225F4F8603B}" name="Preprocessing"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{90C5EED4-AE9B-47F5-AB56-30E37F981507}" name="Tabel8" displayName="Tabel8" ref="A1:A18" totalsRowShown="0" dataDxfId="0">
+  <autoFilter ref="A1:A18" xr:uid="{90C5EED4-AE9B-47F5-AB56-30E37F981507}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{E40DDB4E-ED8E-47F3-B335-AD035D4CF2E0}" name="test" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{E7AAA61B-465F-4F02-AD25-69AC236A203B}" name="Tabel9" displayName="Tabel9" ref="B10:G13" totalsRowShown="0">
+  <autoFilter ref="B10:G13" xr:uid="{E7AAA61B-465F-4F02-AD25-69AC236A203B}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{4A5B7984-8647-44B3-B04F-55B3ACB0FA7E}" name="Target"/>
+    <tableColumn id="2" xr3:uid="{B7C01D19-34B9-4D0C-87D3-AE21442F3B80}" name="Features"/>
+    <tableColumn id="3" xr3:uid="{25DA4F65-FE11-4EAE-8C4F-D20194BF93B6}" name="Hyperparamaters"/>
+    <tableColumn id="4" xr3:uid="{3D80A144-6FB5-4782-9345-FE16E56E4C4A}" name="Resultaten"/>
+    <tableColumn id="5" xr3:uid="{18542178-C908-487A-9C64-E50FE36090D1}" name="Model"/>
+    <tableColumn id="6" xr3:uid="{E0E3C3B9-32D1-4F7C-8D6D-46AA3407B111}" name="Preprocessing"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{B5A62B5C-1B28-4DDB-A297-2C1224F5040A}" name="Tabel10" displayName="Tabel10" ref="B14:G18" totalsRowShown="0">
+  <autoFilter ref="B14:G18" xr:uid="{B5A62B5C-1B28-4DDB-A297-2C1224F5040A}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{A2F1D64A-1F09-4147-B319-D791A5AD4745}" name="Target"/>
+    <tableColumn id="2" xr3:uid="{DE595CB4-CA1C-4B44-B097-1EDD3053B8B5}" name="Features"/>
+    <tableColumn id="3" xr3:uid="{F82C6A4A-F84C-4082-93AB-B1C2C96C07CA}" name="Hyperparamaters"/>
+    <tableColumn id="4" xr3:uid="{CDAED678-19C6-4D12-86AF-9374A6390C49}" name="Resultaten"/>
+    <tableColumn id="5" xr3:uid="{004EB260-254F-407D-93A1-7C147E56D063}" name="Model"/>
+    <tableColumn id="6" xr3:uid="{DC8DDDCB-CDBB-4646-B770-CFD80A25560C}" name="Preprocessing"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -391,63 +515,280 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="46.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="22.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="C8" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="C9" t="s">
         <v>10</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="C13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>0</v>
+      </c>
+      <c r="D14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="C17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="C18" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <tableParts count="5">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>